<commit_message>
clean and comment, add helpers
</commit_message>
<xml_diff>
--- a/inst/extdata/T95_values.xlsx
+++ b/inst/extdata/T95_values.xlsx
@@ -561,7 +561,13 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="21.28515625" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="16.28515625" customWidth="1"/>
     <col min="12" max="12" width="17.28515625" customWidth="1"/>
     <col min="13" max="13" width="16.140625" customWidth="1"/>
   </cols>

</xml_diff>